<commit_message>
Updated data columns description to match revised manuscript
</commit_message>
<xml_diff>
--- a/data/CRM_Data.xlsx
+++ b/data/CRM_Data.xlsx
@@ -5,18 +5,23 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tati\GitHub\mabuyaAnalysis\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Tati\GitHub\mabuyaAnalysis_The_Scientist\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{33815DEB-02C9-4222-A8CF-7AB73674B180}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1014E77B-153F-4C34-BFCA-F005B3FC83FF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="13695" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="ch" sheetId="1" r:id="rId1"/>
     <sheet name="covars" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="152511"/>
+  <extLst>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -167,13 +172,13 @@
     <t>landscape</t>
   </si>
   <si>
-    <t>APA</t>
-  </si>
-  <si>
-    <t>PARNA</t>
-  </si>
-  <si>
     <t>site</t>
+  </si>
+  <si>
+    <t>HPS</t>
+  </si>
+  <si>
+    <t>HPU</t>
   </si>
 </sst>
 </file>
@@ -1622,6 +1627,10 @@
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.46484375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.3984375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="16.53125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.86328125" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="9.86328125" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1648,7 +1657,7 @@
         <v>47</v>
       </c>
       <c r="H1" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" spans="1:10" x14ac:dyDescent="0.45">
@@ -1674,7 +1683,7 @@
         <v>45</v>
       </c>
       <c r="H2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="3" spans="1:10" x14ac:dyDescent="0.45">
@@ -1700,7 +1709,7 @@
         <v>45</v>
       </c>
       <c r="H3" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.45">
@@ -1726,7 +1735,7 @@
         <v>45</v>
       </c>
       <c r="H4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.45">
@@ -1752,7 +1761,7 @@
         <v>45</v>
       </c>
       <c r="H5" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.45">
@@ -1778,7 +1787,7 @@
         <v>45</v>
       </c>
       <c r="H6" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="7" spans="1:10" x14ac:dyDescent="0.45">
@@ -1804,7 +1813,7 @@
         <v>45</v>
       </c>
       <c r="H7" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.45">
@@ -1830,7 +1839,7 @@
         <v>44</v>
       </c>
       <c r="H8" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.45">
@@ -1856,7 +1865,7 @@
         <v>44</v>
       </c>
       <c r="H9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J9" s="1"/>
     </row>
@@ -1883,7 +1892,7 @@
         <v>44</v>
       </c>
       <c r="H10" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J10" s="1"/>
     </row>
@@ -1910,7 +1919,7 @@
         <v>44</v>
       </c>
       <c r="H11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J11" s="1"/>
     </row>
@@ -1937,7 +1946,7 @@
         <v>44</v>
       </c>
       <c r="H12" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J12" s="1"/>
     </row>
@@ -1964,7 +1973,7 @@
         <v>44</v>
       </c>
       <c r="H13" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="J13" s="1"/>
     </row>
@@ -1991,7 +2000,7 @@
         <v>46</v>
       </c>
       <c r="H14" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J14" s="1"/>
     </row>
@@ -2018,7 +2027,7 @@
         <v>46</v>
       </c>
       <c r="H15" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J15" s="1"/>
     </row>
@@ -2045,7 +2054,7 @@
         <v>46</v>
       </c>
       <c r="H16" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="J16" s="1"/>
     </row>
@@ -2072,7 +2081,7 @@
         <v>46</v>
       </c>
       <c r="H17" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.45">
@@ -2098,7 +2107,7 @@
         <v>46</v>
       </c>
       <c r="H18" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.45">
@@ -2124,7 +2133,7 @@
         <v>46</v>
       </c>
       <c r="H19" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.45">
@@ -2150,7 +2159,7 @@
         <v>44</v>
       </c>
       <c r="H20" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.45">
@@ -2176,7 +2185,7 @@
         <v>44</v>
       </c>
       <c r="H21" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.45">
@@ -2202,7 +2211,7 @@
         <v>44</v>
       </c>
       <c r="H22" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.45">
@@ -2228,7 +2237,7 @@
         <v>44</v>
       </c>
       <c r="H23" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.45">
@@ -2254,7 +2263,7 @@
         <v>44</v>
       </c>
       <c r="H24" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.45">
@@ -2280,7 +2289,7 @@
         <v>44</v>
       </c>
       <c r="H25" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.45">
@@ -2306,7 +2315,7 @@
         <v>43</v>
       </c>
       <c r="H26" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.45">
@@ -2332,7 +2341,7 @@
         <v>43</v>
       </c>
       <c r="H27" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.45">
@@ -2358,7 +2367,7 @@
         <v>43</v>
       </c>
       <c r="H28" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.45">
@@ -2384,7 +2393,7 @@
         <v>43</v>
       </c>
       <c r="H29" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.45">
@@ -2410,7 +2419,7 @@
         <v>43</v>
       </c>
       <c r="H30" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.45">
@@ -2436,7 +2445,7 @@
         <v>43</v>
       </c>
       <c r="H31" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.45">
@@ -2462,7 +2471,7 @@
         <v>44</v>
       </c>
       <c r="H32" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.45">
@@ -2488,7 +2497,7 @@
         <v>44</v>
       </c>
       <c r="H33" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.45">
@@ -2514,7 +2523,7 @@
         <v>44</v>
       </c>
       <c r="H34" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.45">
@@ -2540,7 +2549,7 @@
         <v>44</v>
       </c>
       <c r="H35" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.45">
@@ -2566,7 +2575,7 @@
         <v>44</v>
       </c>
       <c r="H36" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.45">
@@ -2592,7 +2601,7 @@
         <v>44</v>
       </c>
       <c r="H37" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.45">
@@ -2618,7 +2627,7 @@
         <v>45</v>
       </c>
       <c r="H38" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.45">
@@ -2644,7 +2653,7 @@
         <v>45</v>
       </c>
       <c r="H39" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.45">
@@ -2670,7 +2679,7 @@
         <v>45</v>
       </c>
       <c r="H40" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.45">
@@ -2696,7 +2705,7 @@
         <v>45</v>
       </c>
       <c r="H41" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.45">
@@ -2722,7 +2731,7 @@
         <v>45</v>
       </c>
       <c r="H42" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.45">
@@ -2748,7 +2757,7 @@
         <v>45</v>
       </c>
       <c r="H43" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.45">
@@ -2774,7 +2783,7 @@
         <v>46</v>
       </c>
       <c r="H44" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.45">
@@ -2800,7 +2809,7 @@
         <v>46</v>
       </c>
       <c r="H45" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.45">
@@ -2826,7 +2835,7 @@
         <v>46</v>
       </c>
       <c r="H46" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.45">
@@ -2852,7 +2861,7 @@
         <v>46</v>
       </c>
       <c r="H47" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.45">
@@ -2878,7 +2887,7 @@
         <v>46</v>
       </c>
       <c r="H48" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.45">
@@ -2904,7 +2913,7 @@
         <v>46</v>
       </c>
       <c r="H49" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>